<commit_message>
refactor(tests): replace hardcoded URLs with ConfigReader in SettingsPage and SensorDashboardPage
</commit_message>
<xml_diff>
--- a/iot-selenium/src/test/resources/testdata/frontend-testing.xlsx
+++ b/iot-selenium/src/test/resources/testdata/frontend-testing.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Bug Report" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Settings &amp; Alerts" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Configuration" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sensor Dashboard" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -21926,4 +21927,1159 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tc_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Test Case Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Feature Ticket #</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Test Scope</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Test Level</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Test Technique</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Test Data Used</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Actual Results</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC-SD01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — traffic data visible after seed</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. POST /api/sensors/generate (Bearer)
+3. Navigate to /home
+4. Wait for #traffic-sensor card to leave loading state
+5. Assert stats row and meta chips visible</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Traffic section (#traffic-sensor) shows readings: meta chips, stats row (Traffic Density, Average Speed, Congestion Level). Not loading or empty state.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>POST /api/sensors/generate; GET /api/sensors/traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC-SD02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — air quality data visible after seed</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. POST /api/sensors/generate
+3. Navigate to /home
+4. Wait for #air-quality-sensor loaded
+5. Assert pollutants / AQI visible</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=air</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Air quality section shows sensor data (meta chips, pollution level / pollutant values). Not loading or empty state.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>POST /api/sensors/generate; GET /api/sensors/air-pollution</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC-SD03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — street light data visible after seed</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. POST /api/sensors/generate
+3. Navigate to /home
+4. Wait for #street-light-sensor loaded
+5. Assert stats row visible</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=street</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Street light section shows Status, Brightness Level, Power Usage stats. Not loading or empty state.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>POST /api/sensors/generate; GET /api/sensors/street-lights</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC-SD07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — empty state traffic after flush</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. DELETE /api/sensors/flush
+3. Navigate to /home
+4. Assert #traffic-sensor empty message</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic;expectedEmpty=No traffic readings available.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Traffic section shows: No traffic readings available.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>DELETE /api/sensors/flush</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC-SD08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — empty state air quality after flush</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. DELETE /api/sensors/flush
+3. On /home assert #air-quality-sensor empty message</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=air;expectedEmpty=No air quality readings available.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Air section shows: No air quality readings available.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>DELETE /api/sensors/flush</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC-SD09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — empty state street light after flush</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. DELETE /api/sensors/flush
+3. On /home assert #street-light-sensor empty message</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=street;expectedEmpty=No street light readings available.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Street section shows: No street light readings available.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>DELETE /api/sensors/flush</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC-SD10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — traffic error state when API unavailable</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Exploratory</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Stop backend or block sensor API
+3. Open /home
+4. Observe #traffic-sensor</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic;expectedError=Unable to load traffic readings right now.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Error panel visible with: Unable to load traffic readings right now.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/traffic</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Manual only — requires backend down or network block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-SD11</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — air quality error state when API unavailable</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Exploratory</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Stop backend or block sensor API
+3. Open /home
+4. Observe #air-quality-sensor</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=air;expectedError=Unable to load air quality readings right now.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Error panel: Unable to load air quality readings right now.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/air-pollution</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Manual only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-SD12</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — street light error state when API unavailable</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Exploratory</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Stop backend or block sensor API
+3. Open /home
+4. Observe #street-light-sensor</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=street;expectedError=Unable to load street light readings right now.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Error panel: Unable to load street light readings right now.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/street-lights</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Manual only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-SD13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — traffic refresh reloads readings</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. On /home wait for traffic stats
+4. Click Refresh in #traffic-sensor
+5. Assert section still shows data (not error/empty)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>After refresh, traffic stats remain visible; no error or empty state.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/traffic</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Locator: #traffic-sensor button[aria-label='Refresh'].</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-SD14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — air quality refresh reloads readings</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. Click Refresh in #air-quality-sensor
+4. Assert data still visible</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=air</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>After refresh, air quality data remains visible.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/air-pollution</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-SD15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — street light refresh reloads readings</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. Click Refresh in #street-light-sensor
+4. Assert stats still visible</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=street</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>After refresh, street light stats remain visible.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/street-lights</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-SD16</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — traffic View Alerts modal open and close</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. Click View traffic alerts in #traffic-sensor
+4. Assert modal backdrop visible
+5. Click Close alerts
+6. Assert modal closed</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Modal opens on View Alerts; closes via button[aria-label='Close alerts']. Backdrop gone.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Locator: #traffic-sensor button[aria-label='View traffic alerts'].</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-SD17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Selenium Sensor Dashboard — air quality View Alerts modal open and close</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. Click View air quality alerts
+4. Assert modal open
+5. Close modal</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=air</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Modal opens and closes for air quality alerts.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Locator: #air-quality-sensor button[aria-label='View air quality alerts'].</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-SD18</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — street light View Alerts button (DOM check)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Visual inspection</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data
+3. Inspect #street-light-sensor actions row in live DOM</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Confirm button.alerts-btn exists and opens modal. Add Selenium row after live DOM sign-off.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Deferred Selenium: template has button.alerts-btn but no aria-label; live DOM verification required before TC-SD19 automation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-SD19</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — traffic history dropdown changes displayed reading</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed data (multiple readings)
+3. Open history select in #traffic-sensor
+4. Select non-zero option if present
+5. Assert stats update</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;section=traffic;historyIndex=1;minHistoryOptions=2</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Selecting another history option updates displayed traffic metrics.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>GET /api/sensors/traffic</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Skip or disable if seed returns single reading only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-SD20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sensor Dashboard — traffic trend chart layout</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Visual inspection</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed traffic data
+3. Inspect trend panel</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Traffic Density Trend bar chart renders correctly.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Manual only — SVG/chart not automated.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(alerts): add data-driven Alerts & Notifications Selenium tests
</commit_message>
<xml_diff>
--- a/iot-selenium/src/test/resources/testdata/frontend-testing.xlsx
+++ b/iot-selenium/src/test/resources/testdata/frontend-testing.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Settings &amp; Alerts" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Configuration" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Sensor Dashboard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Alerts &amp; Notifications" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2383,6 +2384,923 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tc_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Test Case Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Feature Ticket #</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Test Scope</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Test Level</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Test Technique</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Test Data Used</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Actual Results</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC-AN01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — panel opens from bell</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Navigate to /home
+3. Click Notifications bell</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;expectedTitle=Notifications</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Panel visible; header shows Notifications</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Locator: button[aria-label='Notifications']</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC-AN02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — panel closes via close button</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Open notification panel
+3. Click close button</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Panel not visible after close</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Locator: button.close-btn[aria-label='Close notifications']</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC-AN03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — empty state when no alerts</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Ensure no alerts (API list empty)
+3. Open notification panel</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;expectedEmpty=No new notifications</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Empty state text shown; no alert cards in panel</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Delete all alerts via API in test setup when needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC-AN04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — badge hidden when no unread alerts</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Ensure no alerts
+3. Observe bell</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;expectedBadgeVisible=false</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Unread badge (.notify-badge) is not displayed</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC-AN05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — badge visible after alerts seeded</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed sensors and low traffic threshold
+3. Refresh traffic
+4. Open panel</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;thresholdPlaceholder=Enter a value between 0 to 500;thresholdValue=1;minAlertCards=1;expectedBadgeVisible=true</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Unread badge displayed with count &gt;= 1</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>POST /api/sensors/generate; save threshold; refresh traffic sensor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC-AN06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — alert card listed in panel</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed alerts
+3. Open notification panel</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;thresholdPlaceholder=Enter a value between 0 to 500;thresholdValue=1;minAlertCards=1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>At least one alert card with non-blank title and message</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC-AN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — click alert opens traffic sensor modal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed traffic alert
+3. Open panel and click first alert</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;thresholdPlaceholder=Enter a value between 0 to 500;thresholdValue=1;sensorType=traffic</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Panel closes; traffic sensor alerts modal visible</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Expect #traffic-sensor .modal-backdrop</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-AN08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — click alert opens air quality modal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed air alert with ozone threshold
+3. Open panel and click first alert</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;requires=air_quality_threshold;airThresholdPlaceholder=Enter a value between 0 to 300;airThresholdValue=0;minAlertCards=1;sensorType=air-quality</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Panel closes; air quality sensor alerts modal visible</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Set ozone threshold before refresh air sensor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-AN09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — delete alert from traffic modal</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Seed traffic alert
+3. Open panel, jump to traffic modal
+4. Delete first alert</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;thresholdPlaceholder=Enter a value between 0 to 500;thresholdValue=1;section=traffic</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Card removed from modal list</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Locator: #traffic-sensor button[aria-label='Delete alert']</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-AN10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Manual Notifications — toast on new alert</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Visual inspection</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Trigger a new alert after panel initialized</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Toast appears top-right for ~5 seconds</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>MatSnackBar .alert-toast — not Selenium automated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-AN11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manual Notifications — expand detailed report in panel</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Visual inspection</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1. Open panel with alerts</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Detailed report section expands (if UX supports without navigation)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Single click also navigates — manual sign-off only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-AN12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Selenium Notifications — panel available on settings route</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>86c9qjxmf</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1. Log in
+2. Navigate to /settings
+3. Click Notifications bell</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>email=john@example.com;password=Password123!;route=/settings;expectedTitle=Notifications</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Panel visible on settings page</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Topbar includes app-notification-panel on /settings</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>